<commit_message>
feat(dynawo_inputs): read Model Map key and zones from the Excel, drop WECC hardcodes
</commit_message>
<xml_diff>
--- a/tools/dynawo_inputs/examples/WECCSample_full.xlsx
+++ b/tools/dynawo_inputs/examples/WECCSample_full.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Général" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone1a" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REEC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGC" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REPC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Général" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Model Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Zone1a" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Zone3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="REEC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="REGC" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="REPC" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,6 +433,36 @@
           <t>Choix</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Combinaison sélectionnée (clé Model Map)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Zone3 lib</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Zone3 prefix</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Zone1 lib</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Zone1 prefix</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -445,6 +475,36 @@
           <t>REPC_A</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Zone3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>REGC_A|REEC_B|Aucun|Aucun|Aucun|Aucun</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PhotovoltaicsWeccCurrentSource</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>photovoltaics_</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PhotovoltaicsWeccCurrentSourceNoPlantControl</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>photovoltaics_</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -457,6 +517,11 @@
           <t>REEC_B</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -469,6 +534,11 @@
           <t>REGC_A</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -481,6 +551,11 @@
           <t>Aucun</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -493,6 +568,11 @@
           <t>Aucun</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -505,6 +585,11 @@
           <t>Aucun</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -515,6 +600,11 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Aucun</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Zone1;Zone3</t>
         </is>
       </c>
     </row>
@@ -1609,27 +1699,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Parameter</t>
+          <t>Paramètres</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Types</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Valeurs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Base unit</t>
+          <t>Bases pour les pu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Commentaires</t>
         </is>
       </c>
     </row>
@@ -2453,27 +2543,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Parameter</t>
+          <t>Paramètres</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Types</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Valeurs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Base unit</t>
+          <t>Bases pour les pu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Commentaires</t>
         </is>
       </c>
     </row>
@@ -2807,27 +2897,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Parameter</t>
+          <t>Paramètres</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Types</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Valeurs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Base unit</t>
+          <t>Bases pour les pu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Commentaires</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: follow the template's PDR power rows and its OLTC starting tap
</commit_message>
<xml_diff>
--- a/tools/dynawo_inputs/examples/WECCSample_full.xlsx
+++ b/tools/dynawo_inputs/examples/WECCSample_full.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Général" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Model Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Zone1a" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Zone3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="REEC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="REGC" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="REPC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Général" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone1a" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REEC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGC" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REPC" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1057,12 +1057,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Z_cc_LvTr</t>
+          <t>r_TG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>0.0001</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1074,16 +1074,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R_cc_LvTr / X_cc_LvTr</t>
+          <t>Z_cc_TG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.02445</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -1091,16 +1091,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>r_TG</t>
+          <t>R_cc_TG / X_cc_TG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>0.01115</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -1108,16 +1108,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Z_cc_TG</t>
+          <t>Pmax_injection_z1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>0.02445</v>
+        <v>90</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -1125,16 +1125,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R_cc_TG / X_cc_TG</t>
+          <t>Pmax_soutirage_z1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>0.01115</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1142,16 +1142,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pmax_injection_z1</t>
+          <t>Qmax_z1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>MVAr</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1159,16 +1159,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pmax_soutirage_z1</t>
+          <t>Qmin_z1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>-30</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>MVAr</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -1176,16 +1176,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Qmax_z1</t>
+          <t>P_share</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MVAr</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -1193,53 +1193,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Qmin_z1</t>
+          <t>Q_share</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MVAr</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>P_share</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Q_share</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1252,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1358,7 +1324,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pmax_PDR</t>
+          <t>Pmax_injection_PDR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -1376,16 +1342,16 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Qmax_PDR</t>
+          <t>Pmax_soutirage_PDR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MVAr</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1394,12 +1360,12 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Qmin_PDR</t>
+          <t>Qmax_PDR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>-30</v>
+        <v>30</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1409,41 +1375,41 @@
       <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Transformateur principal</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Z_cc_TP</t>
+          <t>Qmin_PDR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>0.12</v>
+        <v>-30</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>MVAr</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Transformateur principal</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R_cc_TP / X_cc_TP</t>
+          <t>Z_cc_TP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>0.01</v>
+        <v>0.12</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1452,12 +1418,12 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>N_prises</t>
+          <t>R_cc_TP / X_cc_TP</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>0.01</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1470,16 +1436,16 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>r_max</t>
+          <t>N_prises</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
-        <v>1.1</v>
+        <v>20</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1488,12 +1454,12 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>r_min</t>
+          <t>r_max</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1503,23 +1469,19 @@
       <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Charge auxiliaire</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Un_A</t>
+          <t>r_min</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>kV</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1528,16 +1490,16 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sn_A</t>
+          <t>r_0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MVA</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1546,34 +1508,35 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>r_TA</t>
+          <t>Tap_0</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Charge auxiliaire</t>
+        </is>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Z_cc_TA</t>
+          <t>Un_A</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
-        <v>1e-06</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>pu</t>
+          <t>kV</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1582,16 +1545,16 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R_cc_TA / X_cc_TA</t>
+          <t>Sn_A</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MVA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1600,7 +1563,7 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P_A</t>
+          <t>r_TA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1609,7 +1572,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1618,16 +1581,16 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Q_A</t>
+          <t>Z_cc_TA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="n">
-        <v>0.5</v>
+        <v>1e-06</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MVAr</t>
+          <t>pu</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1636,12 +1599,12 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>alpha</t>
+          <t>R_cc_TA / X_cc_TA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1654,7 +1617,7 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>beta</t>
+          <t>P_A</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1663,10 +1626,64 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Q_A</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MVAr</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>